<commit_message>
UI navigation polish, maintenance cleanup, and weekly reporting updates
</commit_message>
<xml_diff>
--- a/maintenance/UV_CuringSystem_Maintenance_Tracker_Template.xlsx
+++ b/maintenance/UV_CuringSystem_Maintenance_Tracker_Template.xlsx
@@ -766,8 +766,14 @@
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>1008</v>
+      </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr">

</xml_diff>